<commit_message>
B03: final review fixes to the project and catalogue; engine: non-finite results are #NUM!, FORECAST with no x variance #DIV/0!, approximate match skips headers and blanks, whole columns and rows move when filled, NUMBERVALUE with a decimal comma
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014c1dJBK3AzGGtSQkTXrGFg
</commit_message>
<xml_diff>
--- a/assets/data/study/lantern-shop-workbook.xlsx
+++ b/assets/data/study/lantern-shop-workbook.xlsx
@@ -1228,10 +1228,10 @@
     <t xml:space="preserve">Gift</t>
   </si>
   <si>
-    <t xml:space="preserve">Delivery from</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Charge</t>
+    <t xml:space="preserve">Order from</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delivery</t>
   </si>
   <si>
     <t xml:space="preserve">Size from</t>

</xml_diff>